<commit_message>
BOM update & assembly notes
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zzapa\Desktop\Projekty\elektronika\Ignis-overdrive\overdrive_effect\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zzapa\Desktop\Projekty\elektronika\Ignis-overdrive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F2CD512-B068-4502-AB0C-AFA7048D3640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F94B330-95CC-4F3C-A216-08973AFC4A1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E7AAC61D-D9DA-4331-B906-2A3C8347E67B}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="82">
   <si>
     <t>Reference</t>
   </si>
@@ -278,6 +278,21 @@
   </si>
   <si>
     <t>AWG 22</t>
+  </si>
+  <si>
+    <t>heatshrink</t>
+  </si>
+  <si>
+    <t>&lt;2mm</t>
+  </si>
+  <si>
+    <t>60cm</t>
+  </si>
+  <si>
+    <t>WAGO conector</t>
+  </si>
+  <si>
+    <t>WAGO 221-412*</t>
   </si>
 </sst>
 </file>
@@ -308,7 +323,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -402,21 +417,59 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -751,40 +804,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D454D378-8691-4E30-B73A-1BD2331A43EB}">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="48.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="8" t="s">
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="6" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="10">
+        <v>1</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="11" t="s">
         <v>58</v>
       </c>
     </row>
@@ -792,13 +845,13 @@
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="7">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -806,13 +859,13 @@
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="7">
+        <v>1</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -820,13 +873,13 @@
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2">
-        <v>1</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="B5" s="7">
+        <v>1</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>50</v>
       </c>
     </row>
@@ -834,13 +887,13 @@
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="7">
         <v>2</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -848,13 +901,13 @@
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2">
-        <v>1</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="B7" s="7">
+        <v>1</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -862,13 +915,13 @@
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="2">
-        <v>1</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="B8" s="7">
+        <v>1</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>50</v>
       </c>
     </row>
@@ -876,13 +929,13 @@
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="2">
-        <v>1</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="B9" s="7">
+        <v>1</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>50</v>
       </c>
     </row>
@@ -890,13 +943,13 @@
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="7">
         <v>2</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>48</v>
       </c>
     </row>
@@ -904,13 +957,13 @@
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="7">
         <v>2</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>49</v>
       </c>
     </row>
@@ -918,13 +971,13 @@
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="2">
-        <v>1</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="B12" s="7">
+        <v>1</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>53</v>
       </c>
     </row>
@@ -932,13 +985,13 @@
       <c r="A13" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="2">
-        <v>1</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="B13" s="7">
+        <v>1</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>56</v>
       </c>
     </row>
@@ -946,13 +999,13 @@
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="2">
-        <v>1</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="B14" s="7">
+        <v>1</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>57</v>
       </c>
     </row>
@@ -960,13 +1013,13 @@
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="7">
         <v>2</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>46</v>
       </c>
     </row>
@@ -974,13 +1027,13 @@
       <c r="A16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="7">
         <v>3</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>44</v>
       </c>
     </row>
@@ -988,13 +1041,13 @@
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="2">
-        <v>1</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="B17" s="7">
+        <v>1</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="2" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1002,13 +1055,13 @@
       <c r="A18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="2">
-        <v>1</v>
-      </c>
-      <c r="C18" s="2" t="s">
+      <c r="B18" s="7">
+        <v>1</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="2" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1016,13 +1069,13 @@
       <c r="A19" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="2">
-        <v>1</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="B19" s="7">
+        <v>1</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="2" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1030,13 +1083,13 @@
       <c r="A20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="2">
-        <v>1</v>
-      </c>
-      <c r="C20" s="2" t="s">
+      <c r="B20" s="7">
+        <v>1</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="2" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1044,13 +1097,13 @@
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="7">
         <v>2</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="2" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1058,13 +1111,13 @@
       <c r="A22" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="7">
         <v>3</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="2" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1072,13 +1125,13 @@
       <c r="A23" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="7">
         <v>2</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="2" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1086,13 +1139,13 @@
       <c r="A24" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="7">
         <v>2</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="2" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1100,13 +1153,13 @@
       <c r="A25" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="2">
-        <v>1</v>
-      </c>
-      <c r="C25" s="2" t="s">
+      <c r="B25" s="7">
+        <v>1</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="2" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1114,13 +1167,13 @@
       <c r="A26" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B26" s="2">
-        <v>1</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="B26" s="7">
+        <v>1</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="2" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1128,13 +1181,13 @@
       <c r="A27" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="2">
-        <v>1</v>
-      </c>
-      <c r="C27" s="2" t="s">
+      <c r="B27" s="7">
+        <v>1</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="2" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1142,13 +1195,13 @@
       <c r="A28" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="2">
-        <v>1</v>
-      </c>
-      <c r="C28" s="2" t="s">
+      <c r="B28" s="7">
+        <v>1</v>
+      </c>
+      <c r="C28" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="2" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1156,13 +1209,13 @@
       <c r="A29" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B29" s="2">
-        <v>1</v>
-      </c>
-      <c r="C29" s="2" t="s">
+      <c r="B29" s="7">
+        <v>1</v>
+      </c>
+      <c r="C29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="2" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1170,13 +1223,13 @@
       <c r="A30" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30" s="7">
         <v>9</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1184,28 +1237,56 @@
       <c r="A31" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="7">
         <v>9</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="4" t="s">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="2" t="s">
         <v>76</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B34" s="3">
+        <v>2</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>